<commit_message>
docs: atualiza fluxo (MES + SIM/NAO), base, manual e planilha P1-P4
</commit_message>
<xml_diff>
--- a/data/documentos/Chamados_Incidentes_Abertos.xlsx
+++ b/data/documentos/Chamados_Incidentes_Abertos.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="133">
   <si>
     <t xml:space="preserve">ID Chamado</t>
   </si>
@@ -77,7 +77,7 @@
     <t xml:space="preserve">S/4HANA</t>
   </si>
   <si>
-    <t xml:space="preserve">Pedido de Compra</t>
+    <t xml:space="preserve">SAP MM</t>
   </si>
   <si>
     <t xml:space="preserve">Erro ao liberar PO na ME29N</t>
@@ -86,7 +86,7 @@
     <t xml:space="preserve">Usuario recebe 'estrategia de liberacao nao encontrada' ao liberar o pedido.</t>
   </si>
   <si>
-    <t xml:space="preserve">Alta</t>
+    <t xml:space="preserve">P2 - Urgente</t>
   </si>
   <si>
     <t xml:space="preserve">Em andamento</t>
@@ -110,16 +110,13 @@
     <t xml:space="preserve">ECC</t>
   </si>
   <si>
-    <t xml:space="preserve">Migo / Entrada</t>
-  </si>
-  <si>
     <t xml:space="preserve">Divergencia de quantidade no MIGO</t>
   </si>
   <si>
     <t xml:space="preserve">Entrada de mercadoria (101) com diferenca; suspeita de tolerancia mal parametrizada.</t>
   </si>
   <si>
-    <t xml:space="preserve">Media</t>
+    <t xml:space="preserve">P3 - Medio</t>
   </si>
   <si>
     <t xml:space="preserve">Aberto</t>
@@ -128,9 +125,6 @@
     <t xml:space="preserve">INC0010236</t>
   </si>
   <si>
-    <t xml:space="preserve">Mestre de Materiais</t>
-  </si>
-  <si>
     <t xml:space="preserve">Material bloqueado para movimentacao</t>
   </si>
   <si>
@@ -143,9 +137,6 @@
     <t xml:space="preserve">2026-07-08</t>
   </si>
   <si>
-    <t xml:space="preserve">MIRO / Fatura</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bloqueio de fatura por variacao de preco</t>
   </si>
   <si>
@@ -158,7 +149,7 @@
     <t xml:space="preserve">PP</t>
   </si>
   <si>
-    <t xml:space="preserve">Ordem de Producao</t>
+    <t xml:space="preserve">SAP PP</t>
   </si>
   <si>
     <t xml:space="preserve">Ordem de producao nao confirma</t>
@@ -179,7 +170,7 @@
     <t xml:space="preserve">WM</t>
   </si>
   <si>
-    <t xml:space="preserve">Transferencia</t>
+    <t xml:space="preserve">SAP WM</t>
   </si>
   <si>
     <t xml:space="preserve">Tarefa de WM sem posicao de destino</t>
@@ -188,7 +179,7 @@
     <t xml:space="preserve">LT01 nao determina o deposito de destino.</t>
   </si>
   <si>
-    <t xml:space="preserve">Baixa</t>
+    <t xml:space="preserve">P4 - Leve</t>
   </si>
   <si>
     <t xml:space="preserve">Time WM</t>
@@ -200,7 +191,7 @@
     <t xml:space="preserve">QM</t>
   </si>
   <si>
-    <t xml:space="preserve">Lote de Inspecao</t>
+    <t xml:space="preserve">SAP QM</t>
   </si>
   <si>
     <t xml:space="preserve">Lote de inspecao nao gerado na entrada</t>
@@ -218,9 +209,6 @@
     <t xml:space="preserve">2026-07-10</t>
   </si>
   <si>
-    <t xml:space="preserve">Contrato</t>
-  </si>
-  <si>
     <t xml:space="preserve">Contrato nao aparece na ME21N</t>
   </si>
   <si>
@@ -230,9 +218,6 @@
     <t xml:space="preserve">INC0010242</t>
   </si>
   <si>
-    <t xml:space="preserve">Requisicao de Compra</t>
-  </si>
-  <si>
     <t xml:space="preserve">RC nao converte em PO automaticamente</t>
   </si>
   <si>
@@ -248,7 +233,7 @@
     <t xml:space="preserve">MES</t>
   </si>
   <si>
-    <t xml:space="preserve">Integracao Opcenter</t>
+    <t xml:space="preserve">Integracao/MES</t>
   </si>
   <si>
     <t xml:space="preserve">Falha de integracao SAP x Opcenter</t>
@@ -257,15 +242,15 @@
     <t xml:space="preserve">Ordem nao replica para o MES Opcenter; IDoc em status 51.</t>
   </si>
   <si>
+    <t xml:space="preserve">P1 - Critico</t>
+  </si>
+  <si>
     <t xml:space="preserve">Time Integracao</t>
   </si>
   <si>
     <t xml:space="preserve">INC0010244</t>
   </si>
   <si>
-    <t xml:space="preserve">Integracao PAS-X</t>
-  </si>
-  <si>
     <t xml:space="preserve">Aponto de producao PAS-X nao retorna ao SAP</t>
   </si>
   <si>
@@ -278,9 +263,6 @@
     <t xml:space="preserve">2026-07-13</t>
   </si>
   <si>
-    <t xml:space="preserve">Estoque</t>
-  </si>
-  <si>
     <t xml:space="preserve">Diferenca de estoque apos inventario</t>
   </si>
   <si>
@@ -290,9 +272,6 @@
     <t xml:space="preserve">INC0010246</t>
   </si>
   <si>
-    <t xml:space="preserve">Fornecedor</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fornecedor bloqueado para compras</t>
   </si>
   <si>
@@ -305,9 +284,6 @@
     <t xml:space="preserve">2026-07-14</t>
   </si>
   <si>
-    <t xml:space="preserve">MRP</t>
-  </si>
-  <si>
     <t xml:space="preserve">MRP nao gera necessidades</t>
   </si>
   <si>
@@ -317,9 +293,6 @@
     <t xml:space="preserve">INC0010248</t>
   </si>
   <si>
-    <t xml:space="preserve">Picking</t>
-  </si>
-  <si>
     <t xml:space="preserve">Divergencia no picking da remessa</t>
   </si>
   <si>
@@ -332,9 +305,6 @@
     <t xml:space="preserve">2026-07-15</t>
   </si>
   <si>
-    <t xml:space="preserve">Preco / Condicao</t>
-  </si>
-  <si>
     <t xml:space="preserve">Condicao de preco nao encontrada</t>
   </si>
   <si>
@@ -344,9 +314,6 @@
     <t xml:space="preserve">INC0010250</t>
   </si>
   <si>
-    <t xml:space="preserve">Certificado</t>
-  </si>
-  <si>
     <t xml:space="preserve">Certificado de qualidade nao emitido</t>
   </si>
   <si>
@@ -359,9 +326,6 @@
     <t xml:space="preserve">2026-07-16</t>
   </si>
   <si>
-    <t xml:space="preserve">Migracao</t>
-  </si>
-  <si>
     <t xml:space="preserve">Divergencia pos-migracao ECC x S/4</t>
   </si>
   <si>
@@ -371,9 +335,6 @@
     <t xml:space="preserve">INC0010252</t>
   </si>
   <si>
-    <t xml:space="preserve">Autorizacao</t>
-  </si>
-  <si>
     <t xml:space="preserve">Usuario sem autorizacao para ME21N</t>
   </si>
   <si>
@@ -389,9 +350,6 @@
     <t xml:space="preserve">2026-07-17</t>
   </si>
   <si>
-    <t xml:space="preserve">Lista Tecnica</t>
-  </si>
-  <si>
     <t xml:space="preserve">BOM desatualizada na ordem</t>
   </si>
   <si>
@@ -413,9 +371,6 @@
     <t xml:space="preserve">INC0010255</t>
   </si>
   <si>
-    <t xml:space="preserve">Inventario WM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bloqueio de posicao durante inventario</t>
   </si>
   <si>
@@ -434,13 +389,16 @@
     <t xml:space="preserve">Total de chamados</t>
   </si>
   <si>
-    <t xml:space="preserve">Prioridade Alta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prioridade Media</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prioridade Baixa</t>
+    <t xml:space="preserve">Prioridade P1 - Critico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prioridade P2 - Urgente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prioridade P3 - Medio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prioridade P4 - Leve</t>
   </si>
   <si>
     <t xml:space="preserve">Chamados do modulo MM</t>
@@ -527,7 +485,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -556,6 +514,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6E0B4"/>
         <bgColor rgb="FFBFBFBF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B183"/>
+        <bgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -608,7 +572,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -637,6 +601,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -658,7 +626,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -686,6 +654,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6E0B4"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4B183"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -746,7 +722,7 @@
       <rgbColor rgb="FFC6E0B4"/>
       <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFF4B183"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFF8CBAD"/>
       <rgbColor rgb="FF3366FF"/>
@@ -961,10 +937,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
@@ -1068,19 +1044,19 @@
         <v>27</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>22</v>
@@ -1097,7 +1073,7 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>26</v>
@@ -1109,13 +1085,13 @@
         <v>16</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>20</v>
@@ -1138,10 +1114,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>15</v>
@@ -1150,19 +1126,19 @@
         <v>27</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>22</v>
@@ -1179,37 +1155,37 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="G6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="H6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="K6" s="2" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>23</v>
@@ -1220,34 +1196,34 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="I7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>24</v>
@@ -1261,34 +1237,34 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="G8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="H8" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>16</v>
@@ -1302,10 +1278,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>15</v>
@@ -1314,19 +1290,19 @@
         <v>16</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>22</v>
@@ -1343,10 +1319,10 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>15</v>
@@ -1355,19 +1331,19 @@
         <v>27</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>22</v>
@@ -1384,37 +1360,37 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="H11" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>20</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>23</v>
@@ -1425,37 +1401,37 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>20</v>
+        <v>76</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>72</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>23</v>
@@ -1466,10 +1442,10 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>15</v>
@@ -1478,19 +1454,19 @@
         <v>16</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>84</v>
+        <v>17</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="H13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>22</v>
@@ -1507,10 +1483,10 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>15</v>
@@ -1519,13 +1495,13 @@
         <v>27</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>20</v>
@@ -1548,37 +1524,37 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="H15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="J15" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>23</v>
@@ -1589,34 +1565,34 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>97</v>
+        <v>48</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>24</v>
@@ -1630,10 +1606,10 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>15</v>
@@ -1642,19 +1618,19 @@
         <v>16</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>102</v>
+        <v>17</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="H17" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>22</v>
@@ -1671,34 +1647,34 @@
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>106</v>
+        <v>55</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>24</v>
@@ -1712,10 +1688,10 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>15</v>
@@ -1724,13 +1700,13 @@
         <v>16</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>111</v>
+        <v>17</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>20</v>
@@ -1753,10 +1729,10 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>15</v>
@@ -1765,22 +1741,22 @@
         <v>27</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>115</v>
+        <v>17</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="H20" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="I20" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="J20" s="2" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>16</v>
@@ -1794,34 +1770,34 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>121</v>
+        <v>41</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>24</v>
@@ -1835,10 +1811,10 @@
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>15</v>
@@ -1850,16 +1826,16 @@
         <v>17</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>22</v>
@@ -1876,34 +1852,34 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>129</v>
+        <v>48</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>16</v>
@@ -1933,134 +1909,143 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="B4" s="9" t="n">
+      <c r="A4" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="10" t="n">
         <f aca="false">COUNTA(Chamados_Abertos!A2:A23)</f>
         <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="B5" s="9" t="n">
-        <f aca="false">COUNTIF(Chamados_Abertos!H2:H23,"Alta")</f>
+      <c r="A5" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="10" t="n">
+        <f aca="false">COUNTIF(Chamados_Abertos!H2:H23,"P1*")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <f aca="false">COUNTIF(Chamados_Abertos!H2:H23,"P2*")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <f aca="false">COUNTIF(Chamados_Abertos!H2:H23,"P3*")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <f aca="false">COUNTIF(Chamados_Abertos!H2:H23,"P4*")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B6" s="9" t="n">
-        <f aca="false">COUNTIF(Chamados_Abertos!H2:H23,"Media")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="B7" s="9" t="n">
-        <f aca="false">COUNTIF(Chamados_Abertos!H2:H23,"Baixa")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B8" s="9" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" s="10" t="n">
         <f aca="false">COUNTIF(Chamados_Abertos!C2:C23,"MM")</f>
         <v>12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" s="9" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="10" t="n">
         <f aca="false">COUNTIF(Chamados_Abertos!C2:C23,"PP")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="B10" s="9" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="10" t="n">
         <f aca="false">COUNTIF(Chamados_Abertos!C2:C23,"QM")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="B11" s="9" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="10" t="n">
         <f aca="false">COUNTIF(Chamados_Abertos!C2:C23,"WM")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B12" s="9" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B13" s="10" t="n">
         <f aca="false">COUNTIF(Chamados_Abertos!C2:C23,"MES")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="B13" s="9" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B14" s="10" t="n">
         <f aca="false">COUNTIF(Chamados_Abertos!D2:D23,"ECC")</f>
         <v>9</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="B14" s="9" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15" s="10" t="n">
         <f aca="false">COUNTIF(Chamados_Abertos!D2:D23,"S/4HANA")</f>
         <v>13</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="B15" s="9" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="10" t="n">
         <f aca="false">ROUND(AVERAGE(Chamados_Abertos!K2:K23),1)</f>
-        <v>16.7</v>
+        <v>15.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>